<commit_message>
UPLOAD : Menambahkan file absensi mahasiswa teknik informatika angkatan 2024 ke dalam folder latihan-excel-dasar-byGPT
</commit_message>
<xml_diff>
--- a/belajar-excel-dasar/belajar-excel-dasar-05.xlsx
+++ b/belajar-excel-dasar/belajar-excel-dasar-05.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonovo\OneDrive\ドキュメント\belajar-excel-dasar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonovo\OneDrive\ドキュメント\belajar-excel\belajar-excel-dasar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A61E92-1A7B-4C9D-B873-72742E68B482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380CE134-A3B2-456D-A891-8A6CBA599C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{264D266A-F7A6-42F1-B85E-BAE5544DA2EE}"/>
   </bookViews>
@@ -327,37 +327,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -380,11 +350,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -395,46 +365,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1784,7 +1714,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53D1AE61-BBC4-4524-B683-7510F6648353}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A2:D18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1809,7 +1738,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>1</v>
       </c>
@@ -1823,7 +1752,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>2</v>
       </c>
@@ -1837,7 +1766,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>3</v>
       </c>
@@ -1851,7 +1780,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>4</v>
       </c>
@@ -1865,7 +1794,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>5</v>
       </c>
@@ -1879,7 +1808,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>6</v>
       </c>
@@ -1893,7 +1822,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>7</v>
       </c>
@@ -1907,7 +1836,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>8</v>
       </c>
@@ -1921,7 +1850,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>9</v>
       </c>
@@ -1935,7 +1864,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>10</v>
       </c>
@@ -2021,34 +1950,29 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:D18" xr:uid="{53D1AE61-BBC4-4524-B683-7510F6648353}">
-    <filterColumn colId="0">
-      <customFilters>
-        <customFilter operator="greaterThan" val="10"/>
-      </customFilters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:D18">
       <sortCondition ref="B3:B18"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A4:A18">
-    <cfRule type="cellIs" dxfId="8" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
       <formula>8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C18">
-    <cfRule type="cellIs" dxfId="7" priority="4" operator="equal">
+  <conditionalFormatting sqref="C3:C18">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Laki-laki"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="equal">
-      <formula>"Perempuan"</formula>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"perempuan"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C18">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>"perempuan"</formula>
+  <conditionalFormatting sqref="C4:C18">
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+      <formula>"Laki-laki"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"Laki-laki"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
+      <formula>"Perempuan"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>